<commit_message>
Show Process and Anticipation Q4 only when the coaching question is asked.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/FD Inroads - Lane Changes - text.xlsx
+++ b/FD Inroads - Lane Changes - text.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="690" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="198">
   <si>
     <t>Screen</t>
   </si>
@@ -494,6 +494,12 @@
   </si>
   <si>
     <t>Q3</t>
+  </si>
+  <si>
+    <t>Q4</t>
+  </si>
+  <si>
+    <t>Process and Anticipation, when the coaching question is asked</t>
   </si>
   <si>
     <t>Score row</t>
@@ -990,7 +996,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -2835,21 +2841,21 @@
         <v>156</v>
       </c>
     </row>
-    <row r="109" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" s="2" t="s">
         <v>136</v>
       </c>
       <c r="B109" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C109" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C109" s="2" t="s">
+      <c r="D109" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="E109" s="2" t="s">
         <v>160</v>
-      </c>
-      <c r="D109" s="2" t="s">
-        <v>160</v>
-      </c>
-      <c r="E109" s="2" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="110" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2857,13 +2863,13 @@
         <v>136</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>8</v>
@@ -2874,13 +2880,13 @@
         <v>136</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>8</v>
@@ -2891,13 +2897,13 @@
         <v>136</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C112" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>8</v>
@@ -2908,13 +2914,13 @@
         <v>136</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C113" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>8</v>
@@ -2925,13 +2931,13 @@
         <v>136</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C114" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>8</v>
@@ -2942,13 +2948,13 @@
         <v>136</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>12</v>
+        <v>161</v>
       </c>
       <c r="C115" s="2" t="s">
-        <v>13</v>
+        <v>167</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>13</v>
+        <v>167</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>8</v>
@@ -2956,24 +2962,24 @@
     </row>
     <row r="116" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="2" t="s">
-        <v>166</v>
+        <v>136</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="C116" s="2" t="s">
-        <v>166</v>
+        <v>13</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>166</v>
+        <v>13</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>167</v>
+        <v>8</v>
       </c>
     </row>
     <row r="117" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B117" s="2" t="s">
         <v>36</v>
@@ -2990,112 +2996,112 @@
     </row>
     <row r="118" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B118" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C118" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="C118" s="2" t="s">
+      <c r="D118" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="E118" s="2" t="s">
         <v>171</v>
-      </c>
-      <c r="D118" s="2" t="s">
-        <v>171</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="119" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C119" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="120" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C120" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="121" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C121" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="122" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C122" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="123" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C123" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="124" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="C124" s="2" t="s">
         <v>178</v>
@@ -3104,49 +3110,49 @@
         <v>178</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="125" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C125" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="126" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C126" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="127" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C127" s="2" t="s">
         <v>182</v>
@@ -3155,49 +3161,49 @@
         <v>182</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="128" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C128" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="129" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>36</v>
+        <v>183</v>
       </c>
       <c r="C129" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="130" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>185</v>
+        <v>36</v>
       </c>
       <c r="C130" s="2" t="s">
         <v>186</v>
@@ -3206,143 +3212,160 @@
         <v>186</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="131" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B131" s="2" t="s">
         <v>187</v>
       </c>
       <c r="C131" s="2" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>164</v>
+        <v>188</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="132" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B132" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C132" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B132" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="C132" s="2" t="s">
-        <v>189</v>
-      </c>
       <c r="D132" s="2" t="s">
-        <v>189</v>
+        <v>166</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="133" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B133" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C133" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D133" s="2" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E133" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="134" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B134" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C134" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D134" s="2" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E134" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="135" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B135" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C135" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D135" s="2" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E135" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="136" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B136" s="2" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C136" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D136" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E136" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="137" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B137" s="2" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C137" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D137" s="2" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="E137" s="2" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="138" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="2" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B138" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C138" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A139" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B139" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C138" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="D138" s="2" t="s">
-        <v>195</v>
-      </c>
-      <c r="E138" s="2" t="s">
-        <v>169</v>
+      <c r="C139" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="D139" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="E139" s="2" t="s">
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>